<commit_message>
fix (test): Update DataValidation.xlsx artifact to remove the invalid attribute operator="between"
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Misc/DataValidation.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Misc/DataValidation.xlsx
@@ -500,11 +500,11 @@
       <x:formula1>36526</x:formula1>
       <x:formula2/>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A5:A5">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A5:A5">
       <x:formula1>$C$1:$C$2</x:formula1>
       <x:formula2/>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
       <x:formula1>=YesNo</x:formula1>
       <x:formula2/>
     </x:dataValidation>
@@ -692,7 +692,7 @@
       <x:formula1>36526</x:formula1>
       <x:formula2/>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
       <x:formula1>=YesNo</x:formula1>
       <x:formula2/>
     </x:dataValidation>
@@ -720,7 +720,7 @@
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="">
+        <x14:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="">
           <x14:formula1>
             <xm:f>'Data Validation'!$C$1:$C$2</xm:f>
           </x14:formula1>
@@ -906,7 +906,7 @@
       <x:formula1>36526</x:formula1>
       <x:formula2/>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="" sqref="A6:A6">
       <x:formula1>=YesNo</x:formula1>
       <x:formula2/>
     </x:dataValidation>
@@ -927,7 +927,7 @@
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" errorStyle="stop" operator="between" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="">
+        <x14:dataValidation type="list" errorStyle="stop" allowBlank="1" showDropDown="0" showInputMessage="1" showErrorMessage="1" errorTitle="" error="" promptTitle="" prompt="">
           <x14:formula1>
             <xm:f>'Data Validation'!$C$1:$C$2</xm:f>
           </x14:formula1>

</xml_diff>